<commit_message>
implement letters in main
</commit_message>
<xml_diff>
--- a/Specs/Plotter_Specs.xlsx
+++ b/Specs/Plotter_Specs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heinr\OneDrive\Documents\TU\Mechatronik-und-Instrumentierung\Specs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB1DE00-44B1-4CB8-8CD5-8070E46BEDD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E3A03F-E9F4-4B79-9480-709C76818267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="50">
   <si>
     <t>Max speed</t>
   </si>
@@ -140,12 +140,6 @@
     <t>Empirical value to avoid overshoot and gear slips</t>
   </si>
   <si>
-    <t>24:34</t>
-  </si>
-  <si>
-    <t>19:34</t>
-  </si>
-  <si>
     <t>house, 45° diagonals</t>
   </si>
   <si>
@@ -153,6 +147,42 @@
   </si>
   <si>
     <t>To measure accuracy: draw test pattern at home position and on the other side</t>
+  </si>
+  <si>
+    <t>Star pattern</t>
+  </si>
+  <si>
+    <t>Stift ansetzen, aus der Mitte in 8 Richtungen fahren</t>
+  </si>
+  <si>
+    <t>2,5mm</t>
+  </si>
+  <si>
+    <t>Max. v (XY)</t>
+  </si>
+  <si>
+    <t>Min. v (diagonal)</t>
+  </si>
+  <si>
+    <t>Half step @ 200 pps</t>
+  </si>
+  <si>
+    <t>100 steps XY = 29 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200 steps D = </t>
+  </si>
+  <si>
+    <t>Wiederholbarkeit</t>
+  </si>
+  <si>
+    <t>r=1,25mm</t>
+  </si>
+  <si>
+    <t>Genauigkeit</t>
+  </si>
+  <si>
+    <t>r=1mm</t>
   </si>
 </sst>
 </file>
@@ -658,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -687,18 +717,18 @@
         <v>4</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="O2" t="s">
         <v>33</v>
       </c>
       <c r="P2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
       <c r="H3" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
@@ -706,12 +736,9 @@
         <v>5</v>
       </c>
       <c r="B4" s="2">
-        <f>24/34</f>
-        <v>0.70588235294117652</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>35</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C4" s="3"/>
       <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
@@ -721,12 +748,9 @@
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <f>19/34</f>
-        <v>0.55882352941176472</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>36</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C5" s="4"/>
       <c r="D5" s="1" t="s">
         <v>8</v>
       </c>
@@ -737,11 +761,14 @@
       </c>
       <c r="B6" s="1">
         <f>B4*B5</f>
-        <v>0.39446366782006925</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
+      <c r="H7" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -749,10 +776,16 @@
       </c>
       <c r="B8" s="1">
         <f>B2*B6</f>
-        <v>2.9584775086505193</v>
+        <v>7.5</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
+      </c>
+      <c r="H8" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
@@ -765,6 +798,20 @@
       <c r="C9" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="H9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J10" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="11" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -772,10 +819,13 @@
       </c>
       <c r="B11" s="1">
         <f>B9*PI()*B8/360</f>
-        <v>0.25817586686075294</v>
+        <v>0.6544984694978736</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="H11" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
@@ -784,10 +834,42 @@
       </c>
       <c r="B12" s="1">
         <f>B11/2</f>
-        <v>0.12908793343037647</v>
+        <v>0.3272492347489368</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="H12" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12">
+        <f>29*B1/100</f>
+        <v>58</v>
+      </c>
+      <c r="J12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>42</v>
+      </c>
+      <c r="I13">
+        <f>L13*B1/200</f>
+        <v>41.012193308819761</v>
+      </c>
+      <c r="J13" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" t="s">
+        <v>45</v>
+      </c>
+      <c r="L13">
+        <f>29*SQRT(2)</f>
+        <v>41.012193308819761</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="13.2" x14ac:dyDescent="0.25">
@@ -796,7 +878,7 @@
       </c>
       <c r="B14" s="1">
         <f>B1*B11</f>
-        <v>12.908793343037647</v>
+        <v>130.89969389957471</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>16</v>
@@ -808,7 +890,7 @@
       </c>
       <c r="B15" s="1">
         <f>B12*B1</f>
-        <v>6.4543966715188237</v>
+        <v>65.449846949787357</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>16</v>
@@ -819,7 +901,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>18</v>
@@ -833,7 +915,7 @@
         <v>19</v>
       </c>
       <c r="B18" s="2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>18</v>
@@ -846,9 +928,9 @@
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="1" t="e">
         <f>B14/B17</f>
-        <v>129.08793343037647</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>21</v>
@@ -858,9 +940,9 @@
       <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="1" t="e">
         <f>B15/B17</f>
-        <v>64.543966715188233</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>21</v>
@@ -870,9 +952,9 @@
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="1" t="e">
         <f>B14/B18</f>
-        <v>129.08793343037647</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>21</v>
@@ -882,9 +964,9 @@
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="1" t="e">
         <f>B15/B18</f>
-        <v>64.543966715188233</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>21</v>
@@ -894,9 +976,9 @@
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="1" t="e">
         <f>B20*B17^2/2</f>
-        <v>0.6454396671518825</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>12</v>
@@ -907,9 +989,9 @@
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="1" t="e">
         <f>B21/2*B17^2</f>
-        <v>0.32271983357594125</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>12</v>
@@ -920,9 +1002,9 @@
       <c r="A27" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="1" t="e">
         <f>B22*B18^2/2</f>
-        <v>0.6454396671518825</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>12</v>
@@ -933,9 +1015,9 @@
       <c r="A28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="1" t="e">
         <f>B23/2*B18^2</f>
-        <v>0.32271983357594125</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>12</v>
@@ -967,7 +1049,7 @@
         <v>27</v>
       </c>
       <c r="B32" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C32" s="5"/>
     </row>
@@ -976,7 +1058,8 @@
         <v>28</v>
       </c>
       <c r="B33" s="2">
-        <v>50</v>
+        <f>(12*29)*2</f>
+        <v>696</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>12</v>
@@ -986,9 +1069,9 @@
       <c r="A34" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="1" t="e">
         <f>(B33-B32*(B25+B27))/B14+B32*(B17+B18)</f>
-        <v>4.1733287202995992</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>18</v>
@@ -998,15 +1081,20 @@
       <c r="A35" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="1" t="e">
         <f>(B33-B32*(B28+B26))/B15+B32*(B17+B18)</f>
-        <v>8.0466574405991977</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <f>B33/B15</f>
+        <v>10.634096677628079</v>
+      </c>
+    </row>
     <row r="40" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
     <row r="43" spans="1:3" ht="13.2" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>